<commit_message>
Update Bill Pay test data and fix LoginTest syntax
</commit_message>
<xml_diff>
--- a/parabank-automation (1)/parabank-automation/src/test/resources/testdata/TestData.xlsx
+++ b/parabank-automation (1)/parabank-automation/src/test/resources/testdata/TestData.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RequestLoan" sheetId="1" r:id="R2c4120f675014f24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TransferFunds" sheetId="2" r:id="Rba42f9b5574644f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BillPay" sheetId="3" r:id="Rd673daf3e9b04b36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login" sheetId="4" r:id="R2d7b0d35bde6453b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RequestLoan" sheetId="1" r:id="R07cfbb3697d24cc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TransferFunds" sheetId="2" r:id="Ra6ffdad22a484fa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BillPay" sheetId="3" r:id="R3fb3e6e556dd4bdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login" sheetId="4" r:id="R34e1af2f3ccc4d9b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -61,7 +61,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="40">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -125,6 +125,34 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -596,6 +624,7 @@
     <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -635,6 +664,9 @@
       <x:c r="L1" s="19" t="str">
         <x:v>ExpectedResult</x:v>
       </x:c>
+      <x:c r="M1" s="39" t="str">
+        <x:v>ExpectedMessage</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="24" t="str">
@@ -673,6 +705,7 @@
       <x:c r="L2" s="24" t="str">
         <x:v>Success</x:v>
       </x:c>
+      <x:c r="M2" s="39" t="str"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="24" t="str">
@@ -711,6 +744,9 @@
       <x:c r="L3" s="24" t="str">
         <x:v>AccountMismatch</x:v>
       </x:c>
+      <x:c r="M3" s="39" t="str">
+        <x:v>The account numbers do not match.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="24" t="str">
@@ -749,6 +785,7 @@
       <x:c r="L4" s="24" t="str">
         <x:v>BalanceDeducted</x:v>
       </x:c>
+      <x:c r="M4" s="39" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="24" t="str">
@@ -787,6 +824,7 @@
       <x:c r="L5" s="24" t="str">
         <x:v>TransactionHistory</x:v>
       </x:c>
+      <x:c r="M5" s="39" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="24" t="str">
@@ -823,6 +861,7 @@
       <x:c r="L6" s="24" t="str">
         <x:v>AmountRequired</x:v>
       </x:c>
+      <x:c r="M6" s="39" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add advanced Bill Pay automation scenarios
</commit_message>
<xml_diff>
--- a/parabank-automation (1)/parabank-automation/src/test/resources/testdata/TestData.xlsx
+++ b/parabank-automation (1)/parabank-automation/src/test/resources/testdata/TestData.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RequestLoan" sheetId="1" r:id="R07cfbb3697d24cc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TransferFunds" sheetId="2" r:id="Ra6ffdad22a484fa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BillPay" sheetId="3" r:id="R3fb3e6e556dd4bdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login" sheetId="4" r:id="R34e1af2f3ccc4d9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RequestLoan" sheetId="1" r:id="R94bfbb06b53a4bcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TransferFunds" sheetId="2" r:id="Rd10eed4ab7fc475b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BillPay" sheetId="3" r:id="Rbe47e1113a874a62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login" sheetId="4" r:id="R02feb70d8ff94cc3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -36,12 +36,22 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -61,7 +71,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="40">
+  <x:cellXfs count="59">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -153,6 +163,59 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -612,60 +675,76 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="17" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="25" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="28" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="34" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="23" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="15" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="22" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="18" t="str">
+      <x:c r="A1" s="57" t="str">
         <x:v>TestCaseId</x:v>
       </x:c>
-      <x:c r="B1" s="18" t="str">
+      <x:c r="B1" s="57" t="str">
         <x:v>PayeeName</x:v>
       </x:c>
-      <x:c r="C1" s="18" t="str">
+      <x:c r="C1" s="57" t="str">
         <x:v>Street</x:v>
       </x:c>
-      <x:c r="D1" s="18" t="str">
+      <x:c r="D1" s="57" t="str">
         <x:v>City</x:v>
       </x:c>
-      <x:c r="E1" s="19" t="str">
+      <x:c r="E1" s="51" t="str">
         <x:v>State</x:v>
       </x:c>
-      <x:c r="F1" s="26" t="str">
+      <x:c r="F1" s="58" t="str">
         <x:v>ZipCode</x:v>
       </x:c>
-      <x:c r="G1" s="26" t="str">
+      <x:c r="G1" s="58" t="str">
         <x:v>Phone</x:v>
       </x:c>
-      <x:c r="H1" s="19" t="str">
+      <x:c r="H1" s="51" t="str">
         <x:v>Email</x:v>
       </x:c>
-      <x:c r="I1" s="26" t="str">
+      <x:c r="I1" s="58" t="str">
         <x:v>PayeeAccount</x:v>
       </x:c>
-      <x:c r="J1" s="26" t="str">
+      <x:c r="J1" s="58" t="str">
         <x:v>VerifyAccount</x:v>
       </x:c>
-      <x:c r="K1" s="19" t="str">
+      <x:c r="K1" s="51" t="str">
         <x:v>Amount</x:v>
       </x:c>
-      <x:c r="L1" s="19" t="str">
+      <x:c r="L1" s="51" t="str">
         <x:v>ExpectedResult</x:v>
       </x:c>
-      <x:c r="M1" s="39" t="str">
+      <x:c r="M1" s="51" t="str">
         <x:v>ExpectedMessage</x:v>
+      </x:c>
+      <x:c r="N1" s="51" t="str">
+        <x:v>TestCategory</x:v>
+      </x:c>
+      <x:c r="O1" s="51" t="str">
+        <x:v>AccountType</x:v>
+      </x:c>
+      <x:c r="P1" s="51" t="str">
+        <x:v>SecondPayeeName</x:v>
+      </x:c>
+      <x:c r="Q1" s="51" t="str">
+        <x:v>SecondAmount</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -706,6 +785,12 @@
         <x:v>Success</x:v>
       </x:c>
       <x:c r="M2" s="39" t="str"/>
+      <x:c r="N2" s="39" t="str">
+        <x:v>Smoke/E2E</x:v>
+      </x:c>
+      <x:c r="O2" s="39"/>
+      <x:c r="P2" s="39"/>
+      <x:c r="Q2" s="39"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="24" t="str">
@@ -747,6 +832,12 @@
       <x:c r="M3" s="39" t="str">
         <x:v>The account numbers do not match.</x:v>
       </x:c>
+      <x:c r="N3" s="39" t="str">
+        <x:v>Functional/Negative</x:v>
+      </x:c>
+      <x:c r="O3" s="39"/>
+      <x:c r="P3" s="39"/>
+      <x:c r="Q3" s="39"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="24" t="str">
@@ -786,6 +877,12 @@
         <x:v>BalanceDeducted</x:v>
       </x:c>
       <x:c r="M4" s="39" t="str"/>
+      <x:c r="N4" s="39" t="str">
+        <x:v>Integration</x:v>
+      </x:c>
+      <x:c r="O4" s="39"/>
+      <x:c r="P4" s="39"/>
+      <x:c r="Q4" s="39"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="24" t="str">
@@ -825,6 +922,12 @@
         <x:v>TransactionHistory</x:v>
       </x:c>
       <x:c r="M5" s="39" t="str"/>
+      <x:c r="N5" s="39" t="str">
+        <x:v>Integration/E2E</x:v>
+      </x:c>
+      <x:c r="O5" s="39"/>
+      <x:c r="P5" s="39"/>
+      <x:c r="Q5" s="39"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="24" t="str">
@@ -862,6 +965,223 @@
         <x:v>AmountRequired</x:v>
       </x:c>
       <x:c r="M6" s="39" t="str"/>
+      <x:c r="N6" s="39" t="str">
+        <x:v>Functional/Negative</x:v>
+      </x:c>
+      <x:c r="O6" s="39"/>
+      <x:c r="P6" s="39"/>
+      <x:c r="Q6" s="39"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="39" t="str">
+        <x:v>PB_AUTO_06</x:v>
+      </x:c>
+      <x:c r="B7" s="39" t="str"/>
+      <x:c r="C7" s="39" t="str"/>
+      <x:c r="D7" s="39" t="str"/>
+      <x:c r="E7" s="39" t="str"/>
+      <x:c r="F7" s="39" t="str"/>
+      <x:c r="G7" s="39" t="str"/>
+      <x:c r="H7" s="39" t="str"/>
+      <x:c r="I7" s="39" t="str"/>
+      <x:c r="J7" s="39" t="str"/>
+      <x:c r="K7" s="39" t="str"/>
+      <x:c r="L7" s="39" t="str">
+        <x:v>BillPayFormAndAccountSync</x:v>
+      </x:c>
+      <x:c r="M7" s="39" t="str"/>
+      <x:c r="N7" s="39" t="str">
+        <x:v>Smoke/Regression</x:v>
+      </x:c>
+      <x:c r="O7" s="39" t="str"/>
+      <x:c r="P7" s="39" t="str"/>
+      <x:c r="Q7" s="39" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="39" t="str">
+        <x:v>PB_AUTO_07</x:v>
+      </x:c>
+      <x:c r="B8" s="39" t="str">
+        <x:v>FindTxnPayee</x:v>
+      </x:c>
+      <x:c r="C8" s="39" t="str">
+        <x:v>JP Nagar</x:v>
+      </x:c>
+      <x:c r="D8" s="39" t="str">
+        <x:v>Bangalore</x:v>
+      </x:c>
+      <x:c r="E8" s="39" t="str">
+        <x:v>Karnataka</x:v>
+      </x:c>
+      <x:c r="F8" s="39" t="str">
+        <x:v>560078</x:v>
+      </x:c>
+      <x:c r="G8" s="39" t="str">
+        <x:v>9876543210</x:v>
+      </x:c>
+      <x:c r="H8" s="39" t="str">
+        <x:v>findtxn07@example.com</x:v>
+      </x:c>
+      <x:c r="I8" s="39" t="str">
+        <x:v>154440</x:v>
+      </x:c>
+      <x:c r="J8" s="39" t="str">
+        <x:v>154440</x:v>
+      </x:c>
+      <x:c r="K8" s="39" t="str">
+        <x:v>7.13</x:v>
+      </x:c>
+      <x:c r="L8" s="39" t="str">
+        <x:v>SearchableInFindTransactions</x:v>
+      </x:c>
+      <x:c r="M8" s="39" t="str"/>
+      <x:c r="N8" s="39" t="str">
+        <x:v>Integration/Regression</x:v>
+      </x:c>
+      <x:c r="O8" s="39" t="str"/>
+      <x:c r="P8" s="39" t="str"/>
+      <x:c r="Q8" s="39" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="39" t="str">
+        <x:v>PB_AUTO_08</x:v>
+      </x:c>
+      <x:c r="B9" s="39" t="str">
+        <x:v>NewAccountBillPay</x:v>
+      </x:c>
+      <x:c r="C9" s="39" t="str">
+        <x:v>JP Nagar</x:v>
+      </x:c>
+      <x:c r="D9" s="39" t="str">
+        <x:v>Bangalore</x:v>
+      </x:c>
+      <x:c r="E9" s="39" t="str">
+        <x:v>Karnataka</x:v>
+      </x:c>
+      <x:c r="F9" s="39" t="str">
+        <x:v>560078</x:v>
+      </x:c>
+      <x:c r="G9" s="39" t="str">
+        <x:v>9876543210</x:v>
+      </x:c>
+      <x:c r="H9" s="39" t="str">
+        <x:v>newacct08@example.com</x:v>
+      </x:c>
+      <x:c r="I9" s="39" t="str">
+        <x:v>154440</x:v>
+      </x:c>
+      <x:c r="J9" s="39" t="str">
+        <x:v>154440</x:v>
+      </x:c>
+      <x:c r="K9" s="39" t="str">
+        <x:v>1.17</x:v>
+      </x:c>
+      <x:c r="L9" s="39" t="str">
+        <x:v>NewAccountToBillPayE2E</x:v>
+      </x:c>
+      <x:c r="M9" s="39" t="str"/>
+      <x:c r="N9" s="39" t="str">
+        <x:v>Integration/E2E</x:v>
+      </x:c>
+      <x:c r="O9" s="39" t="str">
+        <x:v>SAVINGS</x:v>
+      </x:c>
+      <x:c r="P9" s="39" t="str"/>
+      <x:c r="Q9" s="39" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="39" t="str">
+        <x:v>PB_AUTO_09</x:v>
+      </x:c>
+      <x:c r="B10" s="39" t="str">
+        <x:v>CumulativePayeeA</x:v>
+      </x:c>
+      <x:c r="C10" s="39" t="str">
+        <x:v>JP Nagar</x:v>
+      </x:c>
+      <x:c r="D10" s="39" t="str">
+        <x:v>Bangalore</x:v>
+      </x:c>
+      <x:c r="E10" s="39" t="str">
+        <x:v>Karnataka</x:v>
+      </x:c>
+      <x:c r="F10" s="39" t="str">
+        <x:v>560078</x:v>
+      </x:c>
+      <x:c r="G10" s="39" t="str">
+        <x:v>9876543210</x:v>
+      </x:c>
+      <x:c r="H10" s="39" t="str">
+        <x:v>cumulative09@example.com</x:v>
+      </x:c>
+      <x:c r="I10" s="39" t="str">
+        <x:v>154440</x:v>
+      </x:c>
+      <x:c r="J10" s="39" t="str">
+        <x:v>154440</x:v>
+      </x:c>
+      <x:c r="K10" s="39" t="str">
+        <x:v>1.21</x:v>
+      </x:c>
+      <x:c r="L10" s="39" t="str">
+        <x:v>CumulativeBalanceAndHistory</x:v>
+      </x:c>
+      <x:c r="M10" s="39" t="str"/>
+      <x:c r="N10" s="39" t="str">
+        <x:v>Integration/Regression</x:v>
+      </x:c>
+      <x:c r="O10" s="39" t="str"/>
+      <x:c r="P10" s="39" t="str">
+        <x:v>CumulativePayeeB</x:v>
+      </x:c>
+      <x:c r="Q10" s="39" t="str">
+        <x:v>1.32</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="39" t="str">
+        <x:v>PB_AUTO_10</x:v>
+      </x:c>
+      <x:c r="B11" s="39" t="str">
+        <x:v>SessionPersistPayee</x:v>
+      </x:c>
+      <x:c r="C11" s="39" t="str">
+        <x:v>JP Nagar</x:v>
+      </x:c>
+      <x:c r="D11" s="39" t="str">
+        <x:v>Bangalore</x:v>
+      </x:c>
+      <x:c r="E11" s="39" t="str">
+        <x:v>Karnataka</x:v>
+      </x:c>
+      <x:c r="F11" s="39" t="str">
+        <x:v>560078</x:v>
+      </x:c>
+      <x:c r="G11" s="39" t="str">
+        <x:v>9876543210</x:v>
+      </x:c>
+      <x:c r="H11" s="39" t="str">
+        <x:v>session10@example.com</x:v>
+      </x:c>
+      <x:c r="I11" s="39" t="str">
+        <x:v>154440</x:v>
+      </x:c>
+      <x:c r="J11" s="39" t="str">
+        <x:v>154440</x:v>
+      </x:c>
+      <x:c r="K11" s="39" t="str">
+        <x:v>1.41</x:v>
+      </x:c>
+      <x:c r="L11" s="39" t="str">
+        <x:v>PersistsAcrossRelogin</x:v>
+      </x:c>
+      <x:c r="M11" s="39" t="str"/>
+      <x:c r="N11" s="39" t="str">
+        <x:v>System/E2E/Regression</x:v>
+      </x:c>
+      <x:c r="O11" s="39" t="str"/>
+      <x:c r="P11" s="39" t="str"/>
+      <x:c r="Q11" s="39" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>